<commit_message>
chore: Projektname ohne s — Defeated by Titan
Beleg: grep nach defeated-by-titans/defeated_by_titans/Defeated by Titans/
       DefeatedByTitans über alle Dateien = 0 Treffer. Excel neu gepackt,
       Integrität ok, 788 Datenzeilen und 12 Blätter unverändert.
Grund: einheitlicher Titel. Betroffen: Crate defeated_by_titan, Fenstertitel
       "Defeated by Titan", Repo defeated-by-titan, Bibel-Dateiname,
       Titel- und Namensschema-Zelle im Backlog.
</commit_message>
<xml_diff>
--- a/gameplay/features.xlsx
+++ b/gameplay/features.xlsx
@@ -45,7 +45,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5698" uniqueCount="2643">
   <si>
-    <t xml:space="preserve">Defeated by Titans — Produktions-Backlog</t>
+    <t xml:space="preserve">Defeated by Titan — Produktions-Backlog</t>
   </si>
   <si>
     <t xml:space="preserve">Vollstaendige To-do-Liste aller Spielfunktionen und Assets. Jede Zeile ist ein Ticket. Zielplattform: PC, Tastatur und Maus, kooperativer Mehrspieler.</t>
@@ -7659,7 +7659,7 @@
     <t xml:space="preserve">Referenzbegriff</t>
   </si>
   <si>
-    <t xml:space="preserve">Defeated by Titans</t>
+    <t xml:space="preserve">Defeated by Titan</t>
   </si>
   <si>
     <t xml:space="preserve">Anmerkung</t>

</xml_diff>